<commit_message>
Updated Process of Analytics page
</commit_message>
<xml_diff>
--- a/Accounting-Analytics-Textbook/Unit 1/data/CostOfLivingByState 2025.xlsx
+++ b/Accounting-Analytics-Textbook/Unit 1/data/CostOfLivingByState 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vican\Documents\GitHub\Accounting-Analytics-Textbook\Accounting-Analytics-Textbook\Unit 1\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FA1B92-C628-4FB8-A6AB-19CA734155EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{940E6758-0F68-4BA2-B05A-B2C4A4E721D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38190" yWindow="0" windowWidth="19410" windowHeight="17280" xr2:uid="{8C834582-AA3D-4554-B932-903DB18D1B7D}"/>
+    <workbookView xWindow="10845" yWindow="180" windowWidth="19410" windowHeight="17280" xr2:uid="{8C834582-AA3D-4554-B932-903DB18D1B7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>Rank</t>
   </si>
@@ -66,168 +66,6 @@
     <t>Misc.</t>
   </si>
   <si>
-    <t>Oklahoma </t>
-  </si>
-  <si>
-    <t>Mississippi </t>
-  </si>
-  <si>
-    <t>Alabama </t>
-  </si>
-  <si>
-    <t>Missouri </t>
-  </si>
-  <si>
-    <t>West Virginia </t>
-  </si>
-  <si>
-    <t>Iowa </t>
-  </si>
-  <si>
-    <t>Kansas </t>
-  </si>
-  <si>
-    <t>Michigan </t>
-  </si>
-  <si>
-    <t>Tennessee </t>
-  </si>
-  <si>
-    <t>Arkansas </t>
-  </si>
-  <si>
-    <t>North Dakota </t>
-  </si>
-  <si>
-    <t>Indiana </t>
-  </si>
-  <si>
-    <t>Kentucky </t>
-  </si>
-  <si>
-    <t>Georgia </t>
-  </si>
-  <si>
-    <t>Texas </t>
-  </si>
-  <si>
-    <t>Nebraska </t>
-  </si>
-  <si>
-    <t>Louisiana </t>
-  </si>
-  <si>
-    <t>Minnesota </t>
-  </si>
-  <si>
-    <t>New Mexico </t>
-  </si>
-  <si>
-    <t>South Carolina </t>
-  </si>
-  <si>
-    <t>Illinois </t>
-  </si>
-  <si>
-    <t>Ohio </t>
-  </si>
-  <si>
-    <t>Montana </t>
-  </si>
-  <si>
-    <t>Wyoming </t>
-  </si>
-  <si>
-    <t>South Dakota </t>
-  </si>
-  <si>
-    <t>Pennsylvania </t>
-  </si>
-  <si>
-    <t>North Carolina </t>
-  </si>
-  <si>
-    <t>Nevada </t>
-  </si>
-  <si>
-    <t>Wisconsin </t>
-  </si>
-  <si>
-    <t>Utah </t>
-  </si>
-  <si>
-    <t>Virginia </t>
-  </si>
-  <si>
-    <t>Idaho </t>
-  </si>
-  <si>
-    <t>Florida </t>
-  </si>
-  <si>
-    <t>Puerto Rico </t>
-  </si>
-  <si>
-    <t>Delaware </t>
-  </si>
-  <si>
-    <t>Colorado </t>
-  </si>
-  <si>
-    <t>Rhode Island </t>
-  </si>
-  <si>
-    <t>New Hampshire </t>
-  </si>
-  <si>
-    <t>Washington </t>
-  </si>
-  <si>
-    <t>Arizona </t>
-  </si>
-  <si>
-    <t>Oregon </t>
-  </si>
-  <si>
-    <t>Maine </t>
-  </si>
-  <si>
-    <t>Connecticut </t>
-  </si>
-  <si>
-    <t>Vermont </t>
-  </si>
-  <si>
-    <t>New Jersey </t>
-  </si>
-  <si>
-    <t>Maryland </t>
-  </si>
-  <si>
-    <t>New York </t>
-  </si>
-  <si>
-    <t>Alaska </t>
-  </si>
-  <si>
-    <t>District of Columbia </t>
-  </si>
-  <si>
-    <t>California </t>
-  </si>
-  <si>
-    <t>Massachusetts </t>
-  </si>
-  <si>
-    <t>Hawaii </t>
-  </si>
-  <si>
-    <t>**</t>
-  </si>
-  <si>
-    <t>U.S.</t>
-  </si>
-  <si>
     <t>Original data source</t>
   </si>
   <si>
@@ -240,23 +78,162 @@
     <t>https://www.kaggle.com/datasets/lukkardata/cost-of-living-missouri-economic-research</t>
   </si>
   <si>
-    <t>I randomized the order of the states.</t>
+    <t>Minnesota</t>
+  </si>
+  <si>
+    <t>Ohio</t>
+  </si>
+  <si>
+    <t>Michigan</t>
+  </si>
+  <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>Arizona</t>
+  </si>
+  <si>
+    <t>Massachusetts</t>
+  </si>
+  <si>
+    <t>Louisiana</t>
+  </si>
+  <si>
+    <t>Maine</t>
+  </si>
+  <si>
+    <t>New Jersey</t>
+  </si>
+  <si>
+    <t>South Dakota</t>
+  </si>
+  <si>
+    <t>North Dakota</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>Rhode Island</t>
+  </si>
+  <si>
+    <t>New Hampshire</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Oklahoma</t>
+  </si>
+  <si>
+    <t>Virginia</t>
+  </si>
+  <si>
+    <t>Connecticut</t>
+  </si>
+  <si>
+    <t>Iowa</t>
+  </si>
+  <si>
+    <t>Maryland</t>
+  </si>
+  <si>
+    <t>South Carolina</t>
+  </si>
+  <si>
+    <t>Tennessee</t>
+  </si>
+  <si>
+    <t>Hawaii</t>
+  </si>
+  <si>
+    <t>Kentucky</t>
+  </si>
+  <si>
+    <t>Missouri</t>
+  </si>
+  <si>
+    <t>Nebraska</t>
+  </si>
+  <si>
+    <t>Pennsylvania</t>
+  </si>
+  <si>
+    <t>Delaware</t>
+  </si>
+  <si>
+    <t>Oregon</t>
+  </si>
+  <si>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Wyoming</t>
+  </si>
+  <si>
+    <t>Arkansas</t>
+  </si>
+  <si>
+    <t>Wisconsin</t>
+  </si>
+  <si>
+    <t>Nevada</t>
+  </si>
+  <si>
+    <t>Vermont</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Alaska</t>
+  </si>
+  <si>
+    <t>Utah</t>
+  </si>
+  <si>
+    <t>New Mexico</t>
+  </si>
+  <si>
+    <t>Kansas</t>
+  </si>
+  <si>
+    <t>Montana</t>
+  </si>
+  <si>
+    <t>Indiana</t>
+  </si>
+  <si>
+    <t>West Virginia</t>
+  </si>
+  <si>
+    <t>Washington</t>
+  </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>Alabama</t>
+  </si>
+  <si>
+    <t>Mississippi</t>
+  </si>
+  <si>
+    <t>Idaho</t>
+  </si>
+  <si>
+    <t>North Carolina</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -291,12 +268,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -316,8 +292,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{43E88935-1FDA-4FAA-B248-D50B9C236CE6}" name="Table2" displayName="Table2" ref="A1:I54" totalsRowShown="0">
-  <autoFilter ref="A1:I54" xr:uid="{43E88935-1FDA-4FAA-B248-D50B9C236CE6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{43E88935-1FDA-4FAA-B248-D50B9C236CE6}" name="Table2" displayName="Table2" ref="A1:I51" totalsRowShown="0">
+  <autoFilter ref="A1:I51" xr:uid="{43E88935-1FDA-4FAA-B248-D50B9C236CE6}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{F80D4532-0D59-4001-B653-FA09A0E02E92}" name="Rank"/>
     <tableColumn id="2" xr3:uid="{861F1316-1A27-40C8-9B44-203CB94E5776}" name="State"/>
@@ -650,7 +626,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECF3EF80-B3C7-46AF-B228-E2B651044CC0}">
-  <dimension ref="A1:I54"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -695,234 +674,234 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C2">
-        <v>99.5</v>
+        <v>93.7</v>
       </c>
       <c r="D2">
-        <v>99.6</v>
+        <v>100.7</v>
       </c>
       <c r="E2">
-        <v>99.7</v>
+        <v>79.8</v>
       </c>
       <c r="F2">
-        <v>92.4</v>
+        <v>95.4</v>
       </c>
       <c r="G2">
-        <v>99.7</v>
+        <v>96.1</v>
       </c>
       <c r="H2">
-        <v>102.5</v>
+        <v>103.1</v>
       </c>
       <c r="I2">
-        <v>100.6</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="C3">
-        <v>109.3</v>
+        <v>95.1</v>
       </c>
       <c r="D3">
-        <v>99</v>
+        <v>99.6</v>
       </c>
       <c r="E3">
-        <v>111.1</v>
+        <v>86.7</v>
       </c>
       <c r="F3">
-        <v>137.5</v>
+        <v>97.1</v>
       </c>
       <c r="G3">
-        <v>96.7</v>
+        <v>99.9</v>
       </c>
       <c r="H3">
-        <v>100.4</v>
+        <v>99.4</v>
       </c>
       <c r="I3">
-        <v>110</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="C4">
-        <v>97.3</v>
+        <v>89.8</v>
       </c>
       <c r="D4">
-        <v>103.4</v>
+        <v>98.9</v>
       </c>
       <c r="E4">
-        <v>94.9</v>
+        <v>73.900000000000006</v>
       </c>
       <c r="F4">
-        <v>87.5</v>
+        <v>97.4</v>
       </c>
       <c r="G4">
-        <v>100.2</v>
+        <v>100.6</v>
       </c>
       <c r="H4">
-        <v>104.9</v>
+        <v>88.4</v>
       </c>
       <c r="I4">
-        <v>97.1</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C5">
-        <v>97</v>
+        <v>94.7</v>
       </c>
       <c r="D5">
-        <v>101.9</v>
+        <v>98.5</v>
       </c>
       <c r="E5">
-        <v>91.2</v>
+        <v>84.8</v>
       </c>
       <c r="F5">
-        <v>90.3</v>
+        <v>97.3</v>
       </c>
       <c r="G5">
-        <v>91.8</v>
+        <v>100</v>
       </c>
       <c r="H5">
-        <v>97.9</v>
+        <v>102.3</v>
       </c>
       <c r="I5">
-        <v>102.6</v>
+        <v>98.1</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6">
-        <v>90.5</v>
+        <v>112.5</v>
       </c>
       <c r="D6">
-        <v>95.1</v>
+        <v>102.5</v>
       </c>
       <c r="E6">
-        <v>79.2</v>
+        <v>134.80000000000001</v>
       </c>
       <c r="F6">
-        <v>92.2</v>
+        <v>106.4</v>
       </c>
       <c r="G6">
-        <v>92.4</v>
+        <v>104.5</v>
       </c>
       <c r="H6">
-        <v>85.4</v>
+        <v>90.8</v>
       </c>
       <c r="I6">
-        <v>97.6</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C7">
-        <v>102</v>
+        <v>145.1</v>
       </c>
       <c r="D7">
-        <v>104.4</v>
+        <v>102.7</v>
       </c>
       <c r="E7">
-        <v>100.2</v>
+        <v>215</v>
       </c>
       <c r="F7">
-        <v>73.900000000000006</v>
+        <v>158.9</v>
       </c>
       <c r="G7">
-        <v>105.3</v>
+        <v>103</v>
       </c>
       <c r="H7">
-        <v>102.8</v>
+        <v>139</v>
       </c>
       <c r="I7">
-        <v>108.3</v>
+        <v>114.6</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8">
-        <v>90.8</v>
+        <v>93.2</v>
       </c>
       <c r="D8">
-        <v>98</v>
+        <v>96.7</v>
       </c>
       <c r="E8">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F8">
-        <v>94.2</v>
+        <v>81.400000000000006</v>
       </c>
       <c r="G8">
-        <v>99.4</v>
+        <v>97.7</v>
       </c>
       <c r="H8">
-        <v>95.2</v>
+        <v>95.6</v>
       </c>
       <c r="I8">
-        <v>96.1</v>
+        <v>100.5</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C9">
-        <v>88</v>
+        <v>113.4</v>
       </c>
       <c r="D9">
-        <v>96.7</v>
+        <v>100.3</v>
       </c>
       <c r="E9">
-        <v>74.8</v>
+        <v>133.19999999999999</v>
       </c>
       <c r="F9">
-        <v>97.5</v>
+        <v>119.8</v>
       </c>
       <c r="G9">
-        <v>87.2</v>
+        <v>104.3</v>
       </c>
       <c r="H9">
-        <v>91</v>
+        <v>117.4</v>
       </c>
       <c r="I9">
-        <v>92.5</v>
+        <v>103.1</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -930,985 +909,985 @@
         <v>44</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C10">
-        <v>113.7</v>
+        <v>114.8</v>
       </c>
       <c r="D10">
-        <v>106.4</v>
+        <v>102.6</v>
       </c>
       <c r="E10">
-        <v>130.69999999999999</v>
+        <v>143.30000000000001</v>
       </c>
       <c r="F10">
-        <v>114.5</v>
+        <v>102.1</v>
       </c>
       <c r="G10">
-        <v>101.2</v>
+        <v>101.4</v>
       </c>
       <c r="H10">
-        <v>113</v>
+        <v>109.2</v>
       </c>
       <c r="I10">
-        <v>106.1</v>
+        <v>104.2</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C11">
-        <v>104</v>
+        <v>97.3</v>
       </c>
       <c r="D11">
-        <v>102.6</v>
+        <v>103.4</v>
       </c>
       <c r="E11">
-        <v>111.4</v>
+        <v>94.9</v>
       </c>
       <c r="F11">
-        <v>88.3</v>
+        <v>87.5</v>
       </c>
       <c r="G11">
-        <v>98.1</v>
+        <v>100.2</v>
       </c>
       <c r="H11">
-        <v>109.1</v>
+        <v>104.9</v>
       </c>
       <c r="I11">
-        <v>103.2</v>
+        <v>97.1</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C12">
-        <v>110.1</v>
+        <v>90.8</v>
       </c>
       <c r="D12">
-        <v>98.8</v>
+        <v>97.2</v>
       </c>
       <c r="E12">
-        <v>116.2</v>
+        <v>76.900000000000006</v>
       </c>
       <c r="F12">
-        <v>120.7</v>
+        <v>84.6</v>
       </c>
       <c r="G12">
-        <v>103</v>
+        <v>97.6</v>
       </c>
       <c r="H12">
-        <v>106.2</v>
+        <v>109.3</v>
       </c>
       <c r="I12">
-        <v>109.9</v>
+        <v>96.6</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C13">
-        <v>89.7</v>
+        <v>91.7</v>
       </c>
       <c r="D13">
-        <v>96.5</v>
+        <v>97.7</v>
       </c>
       <c r="E13">
-        <v>75.599999999999994</v>
+        <v>79.7</v>
       </c>
       <c r="F13">
-        <v>100.4</v>
+        <v>102.6</v>
       </c>
       <c r="G13">
-        <v>90.2</v>
+        <v>97.6</v>
       </c>
       <c r="H13">
-        <v>102.1</v>
+        <v>94.8</v>
       </c>
       <c r="I13">
-        <v>93.9</v>
+        <v>94.5</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C14">
-        <v>91.8</v>
+        <v>109.3</v>
       </c>
       <c r="D14">
-        <v>95.8</v>
+        <v>99</v>
       </c>
       <c r="E14">
-        <v>80</v>
+        <v>111.1</v>
       </c>
       <c r="F14">
-        <v>103.3</v>
+        <v>137.5</v>
       </c>
       <c r="G14">
-        <v>92.1</v>
+        <v>96.7</v>
       </c>
       <c r="H14">
-        <v>98.5</v>
+        <v>100.4</v>
       </c>
       <c r="I14">
-        <v>96.1</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
       </c>
       <c r="C15">
-        <v>93.7</v>
+        <v>110.1</v>
       </c>
       <c r="D15">
-        <v>100.7</v>
+        <v>98.8</v>
       </c>
       <c r="E15">
-        <v>79.8</v>
+        <v>116.2</v>
       </c>
       <c r="F15">
-        <v>95.4</v>
+        <v>120.7</v>
       </c>
       <c r="G15">
-        <v>96.1</v>
+        <v>103</v>
       </c>
       <c r="H15">
-        <v>103.1</v>
+        <v>106.2</v>
       </c>
       <c r="I15">
-        <v>99.8</v>
+        <v>109.9</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C16">
-        <v>100.5</v>
+        <v>102</v>
       </c>
       <c r="D16">
-        <v>98.1</v>
+        <v>105.1</v>
       </c>
       <c r="E16">
-        <v>110.8</v>
+        <v>106</v>
       </c>
       <c r="F16">
-        <v>84.4</v>
+        <v>99.3</v>
       </c>
       <c r="G16">
-        <v>102.1</v>
+        <v>101.2</v>
       </c>
       <c r="H16">
-        <v>89.8</v>
+        <v>90.3</v>
       </c>
       <c r="I16">
-        <v>98.1</v>
+        <v>99.9</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C17">
-        <v>96.4</v>
+        <v>85.5</v>
       </c>
       <c r="D17">
-        <v>104.5</v>
+        <v>95.7</v>
       </c>
       <c r="E17">
-        <v>92.4</v>
+        <v>70.5</v>
       </c>
       <c r="F17">
-        <v>80.400000000000006</v>
+        <v>94.7</v>
       </c>
       <c r="G17">
-        <v>98.5</v>
+        <v>86.7</v>
       </c>
       <c r="H17">
-        <v>105.3</v>
+        <v>94.6</v>
       </c>
       <c r="I17">
-        <v>98.3</v>
+        <v>89.5</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="C18">
-        <v>112</v>
+        <v>101.4</v>
       </c>
       <c r="D18">
-        <v>108.2</v>
+        <v>98.9</v>
       </c>
       <c r="E18">
-        <v>116.8</v>
+        <v>105.2</v>
       </c>
       <c r="F18">
-        <v>96.7</v>
+        <v>98.4</v>
       </c>
       <c r="G18">
-        <v>122.4</v>
+        <v>94.7</v>
       </c>
       <c r="H18">
-        <v>113</v>
+        <v>107.6</v>
       </c>
       <c r="I18">
-        <v>110.7</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="C19">
-        <v>114.9</v>
+        <v>113.5</v>
       </c>
       <c r="D19">
-        <v>105.1</v>
+        <v>101.5</v>
       </c>
       <c r="E19">
-        <v>133.80000000000001</v>
+        <v>120.6</v>
       </c>
       <c r="F19">
-        <v>114.4</v>
+        <v>137.6</v>
       </c>
       <c r="G19">
-        <v>103.6</v>
+        <v>103.1</v>
       </c>
       <c r="H19">
-        <v>105.4</v>
+        <v>112.6</v>
       </c>
       <c r="I19">
-        <v>107.9</v>
+        <v>109.9</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="C20">
-        <v>141.6</v>
+        <v>89.6</v>
       </c>
       <c r="D20">
-        <v>108.8</v>
+        <v>95.7</v>
       </c>
       <c r="E20">
-        <v>197.8</v>
+        <v>77.7</v>
       </c>
       <c r="F20">
-        <v>140.69999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="G20">
-        <v>138.69999999999999</v>
+        <v>95.5</v>
       </c>
       <c r="H20">
-        <v>105.4</v>
+        <v>96</v>
       </c>
       <c r="I20">
-        <v>115.8</v>
+        <v>94.3</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C21">
-        <v>85.5</v>
+        <v>114.9</v>
       </c>
       <c r="D21">
-        <v>95.7</v>
+        <v>105.1</v>
       </c>
       <c r="E21">
-        <v>70.5</v>
+        <v>133.80000000000001</v>
       </c>
       <c r="F21">
-        <v>94.7</v>
+        <v>114.4</v>
       </c>
       <c r="G21">
-        <v>86.7</v>
+        <v>103.6</v>
       </c>
       <c r="H21">
-        <v>94.6</v>
+        <v>105.4</v>
       </c>
       <c r="I21">
-        <v>89.5</v>
+        <v>107.9</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
         <v>33</v>
       </c>
-      <c r="B22" t="s">
-        <v>41</v>
-      </c>
       <c r="C22">
-        <v>102</v>
+        <v>94.6</v>
       </c>
       <c r="D22">
-        <v>105.1</v>
+        <v>98.9</v>
       </c>
       <c r="E22">
-        <v>106</v>
+        <v>84.9</v>
       </c>
       <c r="F22">
-        <v>99.3</v>
+        <v>96.3</v>
       </c>
       <c r="G22">
-        <v>101.2</v>
+        <v>96.1</v>
       </c>
       <c r="H22">
-        <v>90.3</v>
+        <v>95</v>
       </c>
       <c r="I22">
-        <v>99.9</v>
+        <v>99.7</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="C23">
-        <v>135.19999999999999</v>
+        <v>90</v>
       </c>
       <c r="D23">
-        <v>104.5</v>
+        <v>96.7</v>
       </c>
       <c r="E23">
-        <v>200.8</v>
+        <v>81.5</v>
       </c>
       <c r="F23">
-        <v>102.5</v>
+        <v>87.9</v>
       </c>
       <c r="G23">
-        <v>108</v>
+        <v>89.3</v>
       </c>
       <c r="H23">
-        <v>123.6</v>
+        <v>85.9</v>
       </c>
       <c r="I23">
-        <v>111.3</v>
+        <v>95.4</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="C24">
-        <v>87.6</v>
+        <v>182.3</v>
       </c>
       <c r="D24">
-        <v>97.6</v>
+        <v>134.6</v>
       </c>
       <c r="E24">
-        <v>69.099999999999994</v>
+        <v>292.10000000000002</v>
       </c>
       <c r="F24">
-        <v>98.8</v>
+        <v>207</v>
       </c>
       <c r="G24">
-        <v>91.9</v>
+        <v>143.1</v>
       </c>
       <c r="H24">
-        <v>90.7</v>
+        <v>125.9</v>
       </c>
       <c r="I24">
-        <v>94.2</v>
+        <v>124.7</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C25">
-        <v>92.4</v>
+        <v>91.7</v>
       </c>
       <c r="D25">
-        <v>98.9</v>
+        <v>99.7</v>
       </c>
       <c r="E25">
-        <v>78.599999999999994</v>
+        <v>75</v>
       </c>
       <c r="F25">
-        <v>90</v>
+        <v>87.3</v>
       </c>
       <c r="G25">
-        <v>95</v>
+        <v>95.2</v>
       </c>
       <c r="H25">
-        <v>97.3</v>
+        <v>93.3</v>
       </c>
       <c r="I25">
-        <v>100.2</v>
+        <v>101.9</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="C26">
-        <v>127.3</v>
+        <v>88</v>
       </c>
       <c r="D26">
-        <v>130.30000000000001</v>
+        <v>96.7</v>
       </c>
       <c r="E26">
-        <v>131.19999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="F26">
-        <v>132.1</v>
+        <v>97.5</v>
       </c>
       <c r="G26">
-        <v>115.3</v>
+        <v>87.2</v>
       </c>
       <c r="H26">
-        <v>142.1</v>
+        <v>91</v>
       </c>
       <c r="I26">
-        <v>122.7</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C27">
-        <v>112.5</v>
+        <v>92.4</v>
       </c>
       <c r="D27">
-        <v>102.5</v>
+        <v>98.9</v>
       </c>
       <c r="E27">
-        <v>134.80000000000001</v>
+        <v>78.599999999999994</v>
       </c>
       <c r="F27">
-        <v>106.4</v>
+        <v>90</v>
       </c>
       <c r="G27">
-        <v>104.5</v>
+        <v>95</v>
       </c>
       <c r="H27">
-        <v>90.8</v>
+        <v>97.3</v>
       </c>
       <c r="I27">
-        <v>105</v>
+        <v>100.2</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="C28">
-        <v>182.3</v>
+        <v>97.5</v>
       </c>
       <c r="D28">
-        <v>134.6</v>
+        <v>97.4</v>
       </c>
       <c r="E28">
-        <v>292.10000000000002</v>
+        <v>86.8</v>
       </c>
       <c r="F28">
-        <v>207</v>
+        <v>108.5</v>
       </c>
       <c r="G28">
-        <v>143.1</v>
+        <v>104.5</v>
       </c>
       <c r="H28">
-        <v>125.9</v>
+        <v>93.7</v>
       </c>
       <c r="I28">
-        <v>124.7</v>
+        <v>102.5</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C29">
-        <v>89.8</v>
+        <v>103.5</v>
       </c>
       <c r="D29">
-        <v>98.9</v>
+        <v>100.1</v>
       </c>
       <c r="E29">
-        <v>73.900000000000006</v>
+        <v>101.4</v>
       </c>
       <c r="F29">
-        <v>97.4</v>
+        <v>99.4</v>
       </c>
       <c r="G29">
-        <v>100.6</v>
+        <v>100</v>
       </c>
       <c r="H29">
-        <v>88.4</v>
+        <v>106.7</v>
       </c>
       <c r="I29">
-        <v>94.3</v>
+        <v>108.2</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="C30">
-        <v>89.6</v>
+        <v>112.7</v>
       </c>
       <c r="D30">
-        <v>95.7</v>
+        <v>105.1</v>
       </c>
       <c r="E30">
-        <v>77.7</v>
+        <v>131.19999999999999</v>
       </c>
       <c r="F30">
-        <v>89.5</v>
+        <v>94.7</v>
       </c>
       <c r="G30">
-        <v>95.5</v>
+        <v>114.7</v>
       </c>
       <c r="H30">
-        <v>96</v>
+        <v>122.2</v>
       </c>
       <c r="I30">
-        <v>94.3</v>
+        <v>103.3</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C31">
-        <v>94.7</v>
+        <v>104</v>
       </c>
       <c r="D31">
-        <v>98.5</v>
+        <v>102.6</v>
       </c>
       <c r="E31">
-        <v>84.8</v>
+        <v>111.4</v>
       </c>
       <c r="F31">
-        <v>97.3</v>
+        <v>88.3</v>
       </c>
       <c r="G31">
-        <v>100</v>
+        <v>98.1</v>
       </c>
       <c r="H31">
-        <v>102.3</v>
+        <v>109.1</v>
       </c>
       <c r="I31">
-        <v>98.1</v>
+        <v>103.2</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C32">
-        <v>112.7</v>
+        <v>91.8</v>
       </c>
       <c r="D32">
-        <v>105.1</v>
+        <v>95.8</v>
       </c>
       <c r="E32">
-        <v>131.19999999999999</v>
+        <v>80</v>
       </c>
       <c r="F32">
-        <v>94.7</v>
+        <v>103.3</v>
       </c>
       <c r="G32">
-        <v>114.7</v>
+        <v>92.1</v>
       </c>
       <c r="H32">
-        <v>122.2</v>
+        <v>98.5</v>
       </c>
       <c r="I32">
-        <v>103.3</v>
+        <v>96.1</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="B33" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C33">
-        <v>145.1</v>
+        <v>97</v>
       </c>
       <c r="D33">
-        <v>102.7</v>
+        <v>101.9</v>
       </c>
       <c r="E33">
-        <v>215</v>
+        <v>91.2</v>
       </c>
       <c r="F33">
-        <v>158.9</v>
+        <v>90.3</v>
       </c>
       <c r="G33">
-        <v>103</v>
+        <v>91.8</v>
       </c>
       <c r="H33">
-        <v>139</v>
+        <v>97.9</v>
       </c>
       <c r="I33">
-        <v>114.6</v>
+        <v>102.6</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="C34">
-        <v>90</v>
+        <v>90.5</v>
       </c>
       <c r="D34">
-        <v>96.7</v>
+        <v>95.1</v>
       </c>
       <c r="E34">
-        <v>81.5</v>
+        <v>79.2</v>
       </c>
       <c r="F34">
-        <v>87.9</v>
+        <v>92.2</v>
       </c>
       <c r="G34">
-        <v>89.3</v>
+        <v>92.4</v>
       </c>
       <c r="H34">
-        <v>85.9</v>
+        <v>85.4</v>
       </c>
       <c r="I34">
-        <v>95.4</v>
+        <v>97.6</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C35">
-        <v>97.8</v>
+        <v>99.5</v>
       </c>
       <c r="D35">
-        <v>97.7</v>
+        <v>99.6</v>
       </c>
       <c r="E35">
-        <v>94.9</v>
+        <v>99.7</v>
       </c>
       <c r="F35">
-        <v>94.7</v>
+        <v>92.4</v>
       </c>
       <c r="G35">
-        <v>92.9</v>
+        <v>99.7</v>
       </c>
       <c r="H35">
-        <v>110.8</v>
+        <v>102.5</v>
       </c>
       <c r="I35">
-        <v>100.4</v>
+        <v>100.6</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B36" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C36">
-        <v>113.5</v>
+        <v>99.5</v>
       </c>
       <c r="D36">
-        <v>101.5</v>
+        <v>102.9</v>
       </c>
       <c r="E36">
-        <v>120.6</v>
+        <v>111.3</v>
       </c>
       <c r="F36">
-        <v>137.6</v>
+        <v>88.7</v>
       </c>
       <c r="G36">
-        <v>103.1</v>
+        <v>114.4</v>
       </c>
       <c r="H36">
-        <v>112.6</v>
+        <v>85.2</v>
       </c>
       <c r="I36">
-        <v>109.9</v>
+        <v>89.2</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B37" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="C37">
-        <v>93.2</v>
+        <v>113.7</v>
       </c>
       <c r="D37">
-        <v>96.7</v>
+        <v>106.4</v>
       </c>
       <c r="E37">
-        <v>84</v>
+        <v>130.69999999999999</v>
       </c>
       <c r="F37">
-        <v>81.400000000000006</v>
+        <v>114.5</v>
       </c>
       <c r="G37">
-        <v>97.7</v>
+        <v>101.2</v>
       </c>
       <c r="H37">
-        <v>95.6</v>
+        <v>113</v>
       </c>
       <c r="I37">
-        <v>100.5</v>
+        <v>106.1</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C38">
-        <v>103.4</v>
+        <v>124.7</v>
       </c>
       <c r="D38">
-        <v>112.4</v>
+        <v>104.1</v>
       </c>
       <c r="E38">
-        <v>97.5</v>
+        <v>174.2</v>
       </c>
       <c r="F38">
-        <v>170.7</v>
+        <v>100.2</v>
       </c>
       <c r="G38">
-        <v>106.4</v>
+        <v>108.7</v>
       </c>
       <c r="H38">
-        <v>69.5</v>
+        <v>110.5</v>
       </c>
       <c r="I38">
-        <v>91.8</v>
+        <v>105.1</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="B39" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="C39">
-        <v>94.2</v>
+        <v>127.3</v>
       </c>
       <c r="D39">
-        <v>97.9</v>
+        <v>130.30000000000001</v>
       </c>
       <c r="E39">
-        <v>90.2</v>
+        <v>131.19999999999999</v>
       </c>
       <c r="F39">
-        <v>84.1</v>
+        <v>132.1</v>
       </c>
       <c r="G39">
-        <v>92.5</v>
+        <v>115.3</v>
       </c>
       <c r="H39">
-        <v>109.3</v>
+        <v>142.1</v>
       </c>
       <c r="I39">
-        <v>96.6</v>
+        <v>122.7</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C40">
-        <v>101.4</v>
+        <v>100.5</v>
       </c>
       <c r="D40">
-        <v>98.9</v>
+        <v>98.1</v>
       </c>
       <c r="E40">
-        <v>105.2</v>
+        <v>110.8</v>
       </c>
       <c r="F40">
-        <v>98.4</v>
+        <v>84.4</v>
       </c>
       <c r="G40">
-        <v>94.7</v>
+        <v>102.1</v>
       </c>
       <c r="H40">
-        <v>107.6</v>
+        <v>89.8</v>
       </c>
       <c r="I40">
-        <v>101</v>
+        <v>98.1</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B41" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="C41">
-        <v>95.1</v>
+        <v>94.2</v>
       </c>
       <c r="D41">
-        <v>99.6</v>
+        <v>97.9</v>
       </c>
       <c r="E41">
-        <v>86.7</v>
+        <v>90.2</v>
       </c>
       <c r="F41">
-        <v>97.1</v>
+        <v>84.1</v>
       </c>
       <c r="G41">
-        <v>99.9</v>
+        <v>92.5</v>
       </c>
       <c r="H41">
-        <v>99.4</v>
+        <v>109.3</v>
       </c>
       <c r="I41">
-        <v>97.7</v>
+        <v>96.6</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C42">
-        <v>103.5</v>
+        <v>89.7</v>
       </c>
       <c r="D42">
-        <v>100.1</v>
+        <v>96.5</v>
       </c>
       <c r="E42">
-        <v>101.4</v>
+        <v>75.599999999999994</v>
       </c>
       <c r="F42">
-        <v>99.4</v>
+        <v>100.4</v>
       </c>
       <c r="G42">
-        <v>100</v>
+        <v>90.2</v>
       </c>
       <c r="H42">
-        <v>106.7</v>
+        <v>102.1</v>
       </c>
       <c r="I42">
-        <v>108.2</v>
+        <v>93.9</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="B43" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C43">
-        <v>113.4</v>
+        <v>96.4</v>
       </c>
       <c r="D43">
-        <v>100.3</v>
+        <v>104.5</v>
       </c>
       <c r="E43">
-        <v>133.19999999999999</v>
+        <v>92.4</v>
       </c>
       <c r="F43">
-        <v>119.8</v>
+        <v>80.400000000000006</v>
       </c>
       <c r="G43">
-        <v>104.3</v>
+        <v>98.5</v>
       </c>
       <c r="H43">
-        <v>117.4</v>
+        <v>105.3</v>
       </c>
       <c r="I43">
-        <v>103.1</v>
+        <v>98.3</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -1916,356 +1895,269 @@
         <v>11</v>
       </c>
       <c r="B44" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="C44">
         <v>90.8</v>
       </c>
       <c r="D44">
-        <v>97.2</v>
+        <v>98</v>
       </c>
       <c r="E44">
-        <v>76.900000000000006</v>
+        <v>76</v>
       </c>
       <c r="F44">
-        <v>84.6</v>
+        <v>94.2</v>
       </c>
       <c r="G44">
-        <v>97.6</v>
+        <v>99.4</v>
       </c>
       <c r="H44">
-        <v>109.3</v>
+        <v>95.2</v>
       </c>
       <c r="I44">
-        <v>96.6</v>
+        <v>96.1</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B45" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C45">
-        <v>94.6</v>
+        <v>88.6</v>
       </c>
       <c r="D45">
-        <v>98.9</v>
+        <v>96.7</v>
       </c>
       <c r="E45">
-        <v>84.9</v>
+        <v>71.599999999999994</v>
       </c>
       <c r="F45">
-        <v>96.3</v>
+        <v>92.2</v>
       </c>
       <c r="G45">
-        <v>96.1</v>
+        <v>96</v>
       </c>
       <c r="H45">
-        <v>95</v>
+        <v>94.4</v>
       </c>
       <c r="I45">
-        <v>99.7</v>
+        <v>95.4</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C46">
-        <v>114.8</v>
+        <v>112</v>
       </c>
       <c r="D46">
-        <v>102.6</v>
+        <v>108.2</v>
       </c>
       <c r="E46">
-        <v>143.30000000000001</v>
+        <v>116.8</v>
       </c>
       <c r="F46">
-        <v>102.1</v>
+        <v>96.7</v>
       </c>
       <c r="G46">
-        <v>101.4</v>
+        <v>122.4</v>
       </c>
       <c r="H46">
-        <v>109.2</v>
+        <v>113</v>
       </c>
       <c r="I46">
-        <v>104.2</v>
+        <v>110.7</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="C47">
-        <v>91.7</v>
+        <v>141.6</v>
       </c>
       <c r="D47">
-        <v>97.7</v>
+        <v>108.8</v>
       </c>
       <c r="E47">
-        <v>79.7</v>
+        <v>197.8</v>
       </c>
       <c r="F47">
-        <v>102.6</v>
+        <v>140.69999999999999</v>
       </c>
       <c r="G47">
-        <v>97.6</v>
+        <v>138.69999999999999</v>
       </c>
       <c r="H47">
-        <v>94.8</v>
+        <v>105.4</v>
       </c>
       <c r="I47">
-        <v>94.5</v>
+        <v>115.8</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="C48">
-        <v>88.6</v>
+        <v>87.6</v>
       </c>
       <c r="D48">
-        <v>96.7</v>
+        <v>97.6</v>
       </c>
       <c r="E48">
-        <v>71.599999999999994</v>
+        <v>69.099999999999994</v>
       </c>
       <c r="F48">
-        <v>92.2</v>
+        <v>98.8</v>
       </c>
       <c r="G48">
-        <v>96</v>
+        <v>91.9</v>
       </c>
       <c r="H48">
-        <v>94.4</v>
+        <v>90.7</v>
       </c>
       <c r="I48">
-        <v>95.4</v>
+        <v>94.2</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C49" s="1">
-        <v>100</v>
-      </c>
-      <c r="D49" s="1">
-        <v>100</v>
-      </c>
-      <c r="E49" s="1">
-        <v>100</v>
-      </c>
-      <c r="F49" s="1">
-        <v>100</v>
-      </c>
-      <c r="G49" s="1">
-        <v>100</v>
-      </c>
-      <c r="H49" s="1">
-        <v>100</v>
-      </c>
-      <c r="I49" s="1">
-        <v>100</v>
+      <c r="A49">
+        <v>2</v>
+      </c>
+      <c r="B49" t="s">
+        <v>60</v>
+      </c>
+      <c r="C49">
+        <v>87.3</v>
+      </c>
+      <c r="D49">
+        <v>95.9</v>
+      </c>
+      <c r="E49">
+        <v>72.5</v>
+      </c>
+      <c r="F49">
+        <v>89.7</v>
+      </c>
+      <c r="G49">
+        <v>89.5</v>
+      </c>
+      <c r="H49">
+        <v>95.7</v>
+      </c>
+      <c r="I49">
+        <v>93.2</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B50" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="C50">
-        <v>99.5</v>
+        <v>102</v>
       </c>
       <c r="D50">
-        <v>102.9</v>
+        <v>104.4</v>
       </c>
       <c r="E50">
-        <v>111.3</v>
+        <v>100.2</v>
       </c>
       <c r="F50">
-        <v>88.7</v>
+        <v>73.900000000000006</v>
       </c>
       <c r="G50">
-        <v>114.4</v>
+        <v>105.3</v>
       </c>
       <c r="H50">
-        <v>85.2</v>
+        <v>102.8</v>
       </c>
       <c r="I50">
-        <v>89.2</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B51" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="C51">
-        <v>97.5</v>
+        <v>97.8</v>
       </c>
       <c r="D51">
-        <v>97.4</v>
+        <v>97.7</v>
       </c>
       <c r="E51">
-        <v>86.8</v>
+        <v>94.9</v>
       </c>
       <c r="F51">
-        <v>108.5</v>
+        <v>94.7</v>
       </c>
       <c r="G51">
-        <v>104.5</v>
+        <v>92.9</v>
       </c>
       <c r="H51">
-        <v>93.7</v>
+        <v>110.8</v>
       </c>
       <c r="I51">
-        <v>102.5</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>2</v>
-      </c>
-      <c r="B52" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52">
-        <v>87.3</v>
-      </c>
-      <c r="D52">
-        <v>95.9</v>
-      </c>
-      <c r="E52">
-        <v>72.5</v>
-      </c>
-      <c r="F52">
-        <v>89.7</v>
-      </c>
-      <c r="G52">
-        <v>89.5</v>
-      </c>
-      <c r="H52">
-        <v>95.7</v>
-      </c>
-      <c r="I52">
-        <v>93.2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>47</v>
-      </c>
-      <c r="B53" t="s">
-        <v>55</v>
-      </c>
-      <c r="C53">
-        <v>124.7</v>
-      </c>
-      <c r="D53">
-        <v>104.1</v>
-      </c>
-      <c r="E53">
-        <v>174.2</v>
-      </c>
-      <c r="F53">
-        <v>100.2</v>
-      </c>
-      <c r="G53">
-        <v>108.7</v>
-      </c>
-      <c r="H53">
-        <v>110.5</v>
-      </c>
-      <c r="I53">
-        <v>105.1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>13</v>
-      </c>
-      <c r="B54" t="s">
-        <v>21</v>
-      </c>
-      <c r="C54">
-        <v>91.7</v>
-      </c>
-      <c r="D54">
-        <v>99.7</v>
-      </c>
-      <c r="E54">
-        <v>75</v>
-      </c>
-      <c r="F54">
-        <v>87.3</v>
-      </c>
-      <c r="G54">
-        <v>95.2</v>
-      </c>
-      <c r="H54">
-        <v>93.3</v>
-      </c>
-      <c r="I54">
-        <v>101.9</v>
+        <v>100.4</v>
       </c>
     </row>
   </sheetData>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="88" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"+,Bold"&amp;18Cost of Living by State</oddHeader>
+  </headerFooter>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00CC89EF-45F1-4EDE-B2F0-3996473577D6}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>64</v>
+      <c r="A2" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>67</v>
+      <c r="A5" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -2275,4 +2167,10 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{b19c134a-14c9-4d4c-af65-c420f94c8cbb}" enabled="0" method="" siteId="{b19c134a-14c9-4d4c-af65-c420f94c8cbb}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>